<commit_message>
feat: preload menu reference in summary pages and mapping logic
- Integrated the `preloadMenuReference` function into the DailySummaryPage, Index, MonthlySummaryPage, and SummaryPage components to enhance data loading efficiency.
- Updated the `mapRow` utility to utilize the menu reference for improved item normalization and alias handling, ensuring better data consistency across reports.
- Enhanced category and item normalization functions to accommodate new aliasing rules, improving the accuracy of processed data.

This update significantly improves the application's data handling capabilities, providing users with more reliable and consistent reporting outcomes.
</commit_message>
<xml_diff>
--- a/public/VALIDATION DATA.xlsx
+++ b/public/VALIDATION DATA.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026\daily-coffee-ledger\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{19D49150-24EB-455E-A9B2-E61E78C64974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>

</xml_diff>